<commit_message>
Remove __pycache__ files and improve .gitignore
</commit_message>
<xml_diff>
--- a/assets/StatisticalAnalyzer_Excel_Template.xlsx
+++ b/assets/StatisticalAnalyzer_Excel_Template.xlsx
@@ -5,29 +5,41 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pkrumm\Documents\Statistik_dev\BioMedStatX---Code\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pkrumm\Documents\Statistik_dev\BioMedStatX---Code\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BCF053D-8EFA-4ED8-B976-BBF372B155A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51210420-C7EC-4F32-A0FE-9F4DADC3D4B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19320" yWindow="5985" windowWidth="19440" windowHeight="15000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="OneWay" sheetId="1" r:id="rId1"/>
-    <sheet name="Repeated T test" sheetId="8" r:id="rId2"/>
-    <sheet name="Paired" sheetId="2" r:id="rId3"/>
+    <sheet name="T-Test" sheetId="1" r:id="rId1"/>
+    <sheet name="ANOVA" sheetId="9" r:id="rId2"/>
+    <sheet name="Repeated T-test" sheetId="8" r:id="rId3"/>
     <sheet name="RM_1F" sheetId="3" r:id="rId4"/>
-    <sheet name="TwoWay Template" sheetId="4" r:id="rId5"/>
-    <sheet name="TwoWay Test" sheetId="6" r:id="rId6"/>
-    <sheet name="Mixed" sheetId="5" r:id="rId7"/>
-    <sheet name="Datensatz für Poster" sheetId="7" r:id="rId8"/>
+    <sheet name="TwoWay ANOVA" sheetId="6" r:id="rId5"/>
+    <sheet name="Mixed ANOVA" sheetId="5" r:id="rId6"/>
+    <sheet name="Multi-DatasetAnalysis" sheetId="7" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="59">
   <si>
     <t>Group</t>
   </si>
@@ -44,21 +56,12 @@
     <t>Subject</t>
   </si>
   <si>
-    <t>Condition</t>
-  </si>
-  <si>
     <t>S01</t>
   </si>
   <si>
     <t>S02</t>
   </si>
   <si>
-    <t>pre</t>
-  </si>
-  <si>
-    <t>post</t>
-  </si>
-  <si>
     <t>Timepoint</t>
   </si>
   <si>
@@ -74,12 +77,6 @@
     <t>FactorB</t>
   </si>
   <si>
-    <t>Veh</t>
-  </si>
-  <si>
-    <t>Drug</t>
-  </si>
-  <si>
     <t>BetweenGrp</t>
   </si>
   <si>
@@ -158,32 +155,78 @@
     <t>6h</t>
   </si>
   <si>
-    <t>Control</t>
-  </si>
-  <si>
-    <t>Antioxidans A</t>
-  </si>
-  <si>
-    <t>Antioxidans B</t>
-  </si>
-  <si>
-    <t>Messwerte</t>
-  </si>
-  <si>
-    <t>Gruppen</t>
-  </si>
-  <si>
     <t>Before</t>
   </si>
   <si>
     <t>After</t>
+  </si>
+  <si>
+    <t>Sample</t>
+  </si>
+  <si>
+    <t>mArg1 CNRQ</t>
+  </si>
+  <si>
+    <t>WT+WT</t>
+  </si>
+  <si>
+    <t>WT+Nrf2-KO</t>
+  </si>
+  <si>
+    <t>mHO-1 CNRQ</t>
+  </si>
+  <si>
+    <t>mNQ-1 CNRQ</t>
+  </si>
+  <si>
+    <t>NaN</t>
+  </si>
+  <si>
+    <t>mNos2 CNRQ</t>
+  </si>
+  <si>
+    <t>mPDL1 CNRQ</t>
+  </si>
+  <si>
+    <t>Gruppe</t>
+  </si>
+  <si>
+    <t>Messwert</t>
+  </si>
+  <si>
+    <t>ntc</t>
+  </si>
+  <si>
+    <t>keap1</t>
+  </si>
+  <si>
+    <t>wt_wt</t>
+  </si>
+  <si>
+    <t>wt+nrf2ko</t>
+  </si>
+  <si>
+    <t>ntc+wt</t>
+  </si>
+  <si>
+    <t>ntc+nrf2ko</t>
+  </si>
+  <si>
+    <t>keap1+wt</t>
+  </si>
+  <si>
+    <t>keap1+nrf2ko</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="#,##0.00000000"/>
+    <numFmt numFmtId="165" formatCode="#,##0.000"/>
+  </numFmts>
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -214,6 +257,24 @@
       <sz val="10"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9AA83A"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF6089B4"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -223,7 +284,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -246,11 +307,31 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -267,6 +348,31 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -685,6 +791,604 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEFF587B-B563-4293-94E7-9E684D814310}">
+  <dimension ref="A1:B73"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.5703125" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="14">
+        <v>317497.42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="14">
+        <v>268631.01899999997</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="14">
+        <v>211859.378</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="14">
+        <v>205632.54</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" s="14">
+        <v>214881.22399999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" s="14">
+        <v>192811.31200000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" s="14">
+        <v>223875.274</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" s="14">
+        <v>132182.39999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" s="14">
+        <v>261227.54800000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" s="14">
+        <v>140315.93299999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B12" s="14">
+        <v>174263.75899999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B13" s="14">
+        <v>252005.19699999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B14" s="14">
+        <v>188084.73800000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B15" s="14">
+        <v>285774.902</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B16" s="14">
+        <v>239816.19500000001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B17" s="14">
+        <v>233596.87100000001</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="B18" s="14">
+        <v>351397.57799999998</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="B19" s="14">
+        <v>322996.69799999997</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="B20" s="14">
+        <v>211622.304</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="B21" s="14">
+        <v>566549.77099999995</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" s="14">
+        <v>592641.29099999997</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="B23" s="14">
+        <v>673925.14199999999</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="B24" s="14">
+        <v>556283.74699999997</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="B25" s="14">
+        <v>593781.54099999997</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="B26" s="14">
+        <v>562185.70700000005</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="B27" s="14">
+        <v>556721.54099999997</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="B28" s="14">
+        <v>495659.837</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="B29" s="14">
+        <v>494747.902</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="B30" s="14">
+        <v>513508.70899999997</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31" s="14">
+        <v>325469.13</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="B32" s="14">
+        <v>573058.84400000004</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="B33" s="14">
+        <v>541900.79299999995</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B34" s="14">
+        <v>590576.53300000005</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B35" s="14">
+        <v>578878.00899999996</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B36" s="14">
+        <v>457073.26</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B37" s="14">
+        <v>423756.38699999999</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B38" s="14">
+        <v>305208.065</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B39" s="14">
+        <v>253590.75599999999</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B40" s="14">
+        <v>282297.69900000002</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B41" s="14">
+        <v>392604.62199999997</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B42" s="14">
+        <v>399257.95199999999</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B43" s="14">
+        <v>364420.76199999999</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B44" s="14">
+        <v>488414.43699999998</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B45" s="14">
+        <v>407326.261</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B46" s="14">
+        <v>239061.05</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B47" s="14">
+        <v>442695.326</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B48" s="14">
+        <v>427497.00699999998</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B49" s="14">
+        <v>505372.66</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B50" s="14">
+        <v>587377.82900000003</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B51" s="14">
+        <v>700124.54700000002</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B52" s="14">
+        <v>358138.73300000001</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B53" s="14">
+        <v>580047.09900000005</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B54" s="14">
+        <v>593144.28700000001</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B55" s="14">
+        <v>490447.81400000001</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B56" s="14">
+        <v>576824.54799999995</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B57" s="14">
+        <v>444891.76299999998</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B58" s="14">
+        <v>435291.83899999998</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B59" s="14">
+        <v>536366.39199999999</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B60" s="14">
+        <v>516056.38799999998</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B61" s="14">
+        <v>489389.109</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B62" s="14">
+        <v>496422.53</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B63" s="14">
+        <v>609042.57400000002</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B64" s="14">
+        <v>460416.24200000003</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B65" s="14">
+        <v>510136.89600000001</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="B66" s="14">
+        <v>423870.55599999998</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="B67" s="14">
+        <v>414200.36499999999</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="B68" s="14">
+        <v>506687.28399999999</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="B69" s="14">
+        <v>377672.23300000001</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="B70" s="14">
+        <v>237081.601</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="B71" s="14">
+        <v>315259.571</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="B72" s="14">
+        <v>275899.01199999999</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="B73" s="14">
+        <v>318830.84600000002</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32BF23E1-8923-4AB2-B74C-427E6D1071D2}">
   <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -699,7 +1403,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="B2">
         <v>85</v>
@@ -707,7 +1411,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="B3">
         <v>92</v>
@@ -715,7 +1419,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="B4">
         <v>78</v>
@@ -723,7 +1427,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="B5">
         <v>83</v>
@@ -731,7 +1435,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="B6">
         <v>91</v>
@@ -739,7 +1443,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="B7">
         <v>95</v>
@@ -747,7 +1451,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="B8">
         <v>88</v>
@@ -755,7 +1459,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="B9">
         <v>89</v>
@@ -763,7 +1467,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="B10">
         <v>82</v>
@@ -771,120 +1475,10 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="B11">
         <v>88</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2">
-        <v>10.1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3">
-        <v>12.3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4">
-        <v>9.1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5">
-        <v>11.3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6">
-        <v>9.8000000000000007</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7">
-        <v>11.7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8">
-        <v>9.1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9">
-        <v>11.3</v>
       </c>
     </row>
   </sheetData>
@@ -903,7 +1497,7 @@
         <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -911,10 +1505,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C2">
         <v>13</v>
@@ -922,10 +1516,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C3">
         <v>14</v>
@@ -933,10 +1527,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C4">
         <v>15</v>
@@ -944,10 +1538,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -955,10 +1549,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C6">
         <v>4</v>
@@ -966,10 +1560,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C7">
         <v>6</v>
@@ -977,10 +1571,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C8">
         <v>20</v>
@@ -988,10 +1582,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B9" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C9">
         <v>21</v>
@@ -999,10 +1593,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B10" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C10">
         <v>23</v>
@@ -1010,10 +1604,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C11">
         <v>20</v>
@@ -1021,10 +1615,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B12" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C12">
         <v>22</v>
@@ -1032,10 +1626,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B13" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C13">
         <v>20</v>
@@ -1043,10 +1637,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B14" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C14">
         <v>13</v>
@@ -1054,10 +1648,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B15" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C15">
         <v>14</v>
@@ -1065,10 +1659,10 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B16" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C16">
         <v>14</v>
@@ -1076,10 +1670,10 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B17" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C17">
         <v>11</v>
@@ -1087,10 +1681,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B18" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C18">
         <v>9</v>
@@ -1098,10 +1692,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B19" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C19">
         <v>11</v>
@@ -1109,10 +1703,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C20">
         <v>20</v>
@@ -1120,10 +1714,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B21" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C21">
         <v>22</v>
@@ -1131,10 +1725,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B22" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C22">
         <v>20</v>
@@ -1142,10 +1736,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B23" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C23">
         <v>11</v>
@@ -1153,10 +1747,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B24" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C24">
         <v>9</v>
@@ -1164,10 +1758,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B25" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C25">
         <v>11</v>
@@ -1175,10 +1769,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B26" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C26">
         <v>13</v>
@@ -1186,10 +1780,10 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B27" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C27">
         <v>14</v>
@@ -1197,10 +1791,10 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B28" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="C28">
         <v>14</v>
@@ -1213,678 +1807,6 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:C64"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2">
-        <v>1.1100000000000001</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3">
-        <v>2.0299999999999998</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4">
-        <v>1.35</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5">
-        <v>4.22</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="3"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="3"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="3"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B11" t="s">
-        <v>39</v>
-      </c>
-      <c r="C11" s="4">
-        <v>1.843</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B12" t="s">
-        <v>39</v>
-      </c>
-      <c r="C12" s="4">
-        <v>1.9750000000000001</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B13" t="s">
-        <v>39</v>
-      </c>
-      <c r="C13" s="4">
-        <v>2.097</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B14" t="s">
-        <v>39</v>
-      </c>
-      <c r="C14" s="4">
-        <v>2.0819999999999999</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B15" t="s">
-        <v>39</v>
-      </c>
-      <c r="C15" s="4">
-        <v>2.052</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B16" t="s">
-        <v>39</v>
-      </c>
-      <c r="C16" s="4">
-        <v>1.1639999999999999</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B17" t="s">
-        <v>40</v>
-      </c>
-      <c r="C17" s="4">
-        <v>1.8620000000000001</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B18" t="s">
-        <v>40</v>
-      </c>
-      <c r="C18" s="4">
-        <v>3.173</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B19" t="s">
-        <v>40</v>
-      </c>
-      <c r="C19" s="4">
-        <v>3.12</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B20" t="s">
-        <v>40</v>
-      </c>
-      <c r="C20" s="4">
-        <v>4.0720000000000001</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B21" t="s">
-        <v>40</v>
-      </c>
-      <c r="C21" s="4">
-        <v>1.7230000000000001</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B22" t="s">
-        <v>40</v>
-      </c>
-      <c r="C22" s="4">
-        <v>2.0579999999999998</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B23" t="s">
-        <v>41</v>
-      </c>
-      <c r="C23" s="4">
-        <v>1.974</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B24" t="s">
-        <v>41</v>
-      </c>
-      <c r="C24" s="4">
-        <v>1.895</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B25" t="s">
-        <v>41</v>
-      </c>
-      <c r="C25" s="4">
-        <v>2.4260000000000002</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B26" t="s">
-        <v>41</v>
-      </c>
-      <c r="C26" s="4">
-        <v>2.2629999999999999</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B27" t="s">
-        <v>41</v>
-      </c>
-      <c r="C27" s="4">
-        <v>1.5609999999999999</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B28" t="s">
-        <v>41</v>
-      </c>
-      <c r="C28" s="4">
-        <v>1.696</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B29" t="s">
-        <v>39</v>
-      </c>
-      <c r="C29" s="4">
-        <v>0.61519999999999997</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B30" t="s">
-        <v>39</v>
-      </c>
-      <c r="C30" s="4">
-        <v>0.47320000000000001</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B31" t="s">
-        <v>39</v>
-      </c>
-      <c r="C31" s="4">
-        <v>0.63319999999999999</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B32" t="s">
-        <v>39</v>
-      </c>
-      <c r="C32" s="4">
-        <v>0.96350000000000002</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B33" t="s">
-        <v>39</v>
-      </c>
-      <c r="C33" s="4">
-        <v>1.087</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B34" t="s">
-        <v>39</v>
-      </c>
-      <c r="C34" s="4">
-        <v>2.4180000000000001</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B35" t="s">
-        <v>40</v>
-      </c>
-      <c r="C35" s="4">
-        <v>2.222</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B36" t="s">
-        <v>40</v>
-      </c>
-      <c r="C36" s="4">
-        <v>1.923</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B37" t="s">
-        <v>40</v>
-      </c>
-      <c r="C37" s="4">
-        <v>1.9770000000000001</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B38" t="s">
-        <v>40</v>
-      </c>
-      <c r="C38" s="4">
-        <v>3.6440000000000001</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B39" t="s">
-        <v>40</v>
-      </c>
-      <c r="C39" s="4">
-        <v>3.4009999999999998</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B40" t="s">
-        <v>40</v>
-      </c>
-      <c r="C40" s="4">
-        <v>4.141</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B41" t="s">
-        <v>41</v>
-      </c>
-      <c r="C41" s="4">
-        <v>2.024</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B42" t="s">
-        <v>41</v>
-      </c>
-      <c r="C42" s="4">
-        <v>2.4889999999999999</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B43" t="s">
-        <v>41</v>
-      </c>
-      <c r="C43" s="4">
-        <v>3.5630000000000002</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B44" t="s">
-        <v>41</v>
-      </c>
-      <c r="C44" s="4">
-        <v>4.3150000000000004</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B45" t="s">
-        <v>41</v>
-      </c>
-      <c r="C45" s="4">
-        <v>4.1619999999999999</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B46" t="s">
-        <v>41</v>
-      </c>
-      <c r="C46" s="4">
-        <v>4.1559999999999997</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B47" t="s">
-        <v>39</v>
-      </c>
-      <c r="C47" s="4">
-        <v>0.61619999999999997</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A48" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B48" t="s">
-        <v>39</v>
-      </c>
-      <c r="C48" s="4">
-        <v>1.3660000000000001</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B49" t="s">
-        <v>39</v>
-      </c>
-      <c r="C49" s="4">
-        <v>0.35899999999999999</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B50" t="s">
-        <v>39</v>
-      </c>
-      <c r="C50" s="4">
-        <v>1.571</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B51" t="s">
-        <v>39</v>
-      </c>
-      <c r="C51" s="4">
-        <v>1.734</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B52" t="s">
-        <v>39</v>
-      </c>
-      <c r="C52" s="4">
-        <v>1.214</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B53" t="s">
-        <v>40</v>
-      </c>
-      <c r="C53" s="4">
-        <v>2.0009999999999999</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B54" t="s">
-        <v>40</v>
-      </c>
-      <c r="C54" s="4">
-        <v>2.3650000000000002</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B55" t="s">
-        <v>40</v>
-      </c>
-      <c r="C55" s="4">
-        <v>2.5750000000000002</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B56" t="s">
-        <v>40</v>
-      </c>
-      <c r="C56" s="4">
-        <v>3.41</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B57" t="s">
-        <v>40</v>
-      </c>
-      <c r="C57" s="4">
-        <v>3.6850000000000001</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A58" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B58" t="s">
-        <v>40</v>
-      </c>
-      <c r="C58" s="4">
-        <v>3.4969999999999999</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A59" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B59" t="s">
-        <v>41</v>
-      </c>
-      <c r="C59" s="4">
-        <v>2.6930000000000001</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A60" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B60" t="s">
-        <v>41</v>
-      </c>
-      <c r="C60" s="4">
-        <v>1.952</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A61" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B61" t="s">
-        <v>41</v>
-      </c>
-      <c r="C61" s="4">
-        <v>1.579</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A62" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B62" t="s">
-        <v>41</v>
-      </c>
-      <c r="C62" s="4">
-        <v>3.66</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A63" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B63" t="s">
-        <v>41</v>
-      </c>
-      <c r="C63" s="4">
-        <v>3.5369999999999999</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A64" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B64" t="s">
-        <v>41</v>
-      </c>
-      <c r="C64" s="4">
-        <v>3.6659999999999999</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE2D111A-A709-4CD9-B8AF-EA86CA23B91A}">
   <dimension ref="A1:C55"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1896,10 +1818,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -1907,10 +1829,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B2" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C2" s="4">
         <v>1.843</v>
@@ -1918,10 +1840,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B3" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C3" s="4">
         <v>1.9750000000000001</v>
@@ -1929,10 +1851,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B4" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C4" s="4">
         <v>2.097</v>
@@ -1940,10 +1862,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B5" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C5" s="4">
         <v>2.0819999999999999</v>
@@ -1951,10 +1873,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B6" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C6" s="4">
         <v>2.052</v>
@@ -1962,10 +1884,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C7" s="4">
         <v>1.1639999999999999</v>
@@ -1973,10 +1895,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C8" s="4">
         <v>1.8620000000000001</v>
@@ -1984,10 +1906,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B9" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C9" s="4">
         <v>3.173</v>
@@ -1995,10 +1917,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B10" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C10" s="4">
         <v>3.12</v>
@@ -2006,10 +1928,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C11" s="4">
         <v>4.0720000000000001</v>
@@ -2017,10 +1939,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C12" s="4">
         <v>1.7230000000000001</v>
@@ -2028,10 +1950,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B13" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C13" s="4">
         <v>2.0579999999999998</v>
@@ -2039,10 +1961,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14" t="s">
         <v>36</v>
-      </c>
-      <c r="B14" t="s">
-        <v>41</v>
       </c>
       <c r="C14" s="4">
         <v>1.974</v>
@@ -2050,10 +1972,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B15" t="s">
         <v>36</v>
-      </c>
-      <c r="B15" t="s">
-        <v>41</v>
       </c>
       <c r="C15" s="4">
         <v>1.895</v>
@@ -2061,10 +1983,10 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" t="s">
         <v>36</v>
-      </c>
-      <c r="B16" t="s">
-        <v>41</v>
       </c>
       <c r="C16" s="4">
         <v>2.4260000000000002</v>
@@ -2072,10 +1994,10 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" t="s">
         <v>36</v>
-      </c>
-      <c r="B17" t="s">
-        <v>41</v>
       </c>
       <c r="C17" s="4">
         <v>2.2629999999999999</v>
@@ -2083,10 +2005,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" t="s">
         <v>36</v>
-      </c>
-      <c r="B18" t="s">
-        <v>41</v>
       </c>
       <c r="C18" s="4">
         <v>1.5609999999999999</v>
@@ -2094,10 +2016,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B19" t="s">
         <v>36</v>
-      </c>
-      <c r="B19" t="s">
-        <v>41</v>
       </c>
       <c r="C19" s="4">
         <v>1.696</v>
@@ -2105,10 +2027,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B20" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C20" s="4">
         <v>0.61519999999999997</v>
@@ -2116,10 +2038,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B21" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C21" s="4">
         <v>0.47320000000000001</v>
@@ -2127,10 +2049,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B22" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C22" s="4">
         <v>0.63319999999999999</v>
@@ -2138,10 +2060,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B23" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C23" s="4">
         <v>0.96350000000000002</v>
@@ -2149,10 +2071,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B24" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C24" s="4">
         <v>1.087</v>
@@ -2160,10 +2082,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B25" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C25" s="4">
         <v>2.4180000000000001</v>
@@ -2171,10 +2093,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B26" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C26" s="4">
         <v>2.222</v>
@@ -2182,10 +2104,10 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B27" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C27" s="4">
         <v>1.923</v>
@@ -2193,10 +2115,10 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B28" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C28" s="4">
         <v>1.9770000000000001</v>
@@ -2204,10 +2126,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B29" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C29" s="4">
         <v>3.6440000000000001</v>
@@ -2215,10 +2137,10 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B30" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C30" s="4">
         <v>3.4009999999999998</v>
@@ -2226,10 +2148,10 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B31" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C31" s="4">
         <v>4.141</v>
@@ -2237,10 +2159,10 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B32" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C32" s="4">
         <v>2.024</v>
@@ -2248,10 +2170,10 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C33" s="4">
         <v>2.4889999999999999</v>
@@ -2259,10 +2181,10 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C34" s="4">
         <v>3.5630000000000002</v>
@@ -2270,10 +2192,10 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B35" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C35" s="4">
         <v>4.3150000000000004</v>
@@ -2281,10 +2203,10 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B36" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C36" s="4">
         <v>4.1619999999999999</v>
@@ -2292,10 +2214,10 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B37" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C37" s="4">
         <v>4.1559999999999997</v>
@@ -2303,10 +2225,10 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B38" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C38" s="4">
         <v>0.61619999999999997</v>
@@ -2314,10 +2236,10 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B39" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C39" s="4">
         <v>1.3660000000000001</v>
@@ -2325,10 +2247,10 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B40" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C40" s="4">
         <v>0.35899999999999999</v>
@@ -2336,10 +2258,10 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B41" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C41" s="4">
         <v>1.571</v>
@@ -2347,10 +2269,10 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B42" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C42" s="4">
         <v>1.734</v>
@@ -2358,10 +2280,10 @@
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B43" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C43" s="4">
         <v>1.214</v>
@@ -2369,10 +2291,10 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B44" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C44" s="4">
         <v>2.0009999999999999</v>
@@ -2380,10 +2302,10 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B45" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C45" s="4">
         <v>2.3650000000000002</v>
@@ -2391,10 +2313,10 @@
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B46" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C46" s="4">
         <v>2.5750000000000002</v>
@@ -2402,10 +2324,10 @@
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B47" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C47" s="4">
         <v>3.41</v>
@@ -2413,10 +2335,10 @@
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B48" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C48" s="4">
         <v>3.6850000000000001</v>
@@ -2424,10 +2346,10 @@
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B49" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C49" s="4">
         <v>3.4969999999999999</v>
@@ -2435,10 +2357,10 @@
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B50" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C50" s="4">
         <v>2.6930000000000001</v>
@@ -2446,10 +2368,10 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B51" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C51" s="4">
         <v>1.952</v>
@@ -2457,10 +2379,10 @@
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B52" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C52" s="4">
         <v>1.579</v>
@@ -2468,10 +2390,10 @@
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B53" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C53" s="4">
         <v>3.66</v>
@@ -2479,10 +2401,10 @@
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B54" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C54" s="4">
         <v>3.5369999999999999</v>
@@ -2490,10 +2412,10 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B55" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C55" s="4">
         <v>3.6659999999999999</v>
@@ -2505,7 +2427,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D43"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2521,10 +2443,10 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="C1" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
@@ -2532,13 +2454,13 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D2">
         <v>9.8000000000000007</v>
@@ -2546,13 +2468,13 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D3">
         <v>12.7</v>
@@ -2560,13 +2482,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B4" t="s">
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D4">
         <v>10.4</v>
@@ -2574,13 +2496,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B5" t="s">
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D5">
         <v>13.1</v>
@@ -2588,13 +2510,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
         <v>2</v>
       </c>
       <c r="C6" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D6">
         <v>11.9</v>
@@ -2602,13 +2524,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
         <v>2</v>
       </c>
       <c r="C7" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D7">
         <v>15.4</v>
@@ -2616,13 +2538,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
         <v>3</v>
       </c>
       <c r="C8" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D8">
         <v>10.199999999999999</v>
@@ -2630,13 +2552,13 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s">
         <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D9">
         <v>14.3</v>
@@ -2644,13 +2566,13 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B10" t="s">
         <v>3</v>
       </c>
       <c r="C10" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D10">
         <v>11.5</v>
@@ -2658,13 +2580,13 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B11" t="s">
         <v>3</v>
       </c>
       <c r="C11" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D11">
         <v>15</v>
@@ -2672,13 +2594,13 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="B12" t="s">
         <v>3</v>
       </c>
       <c r="C12" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D12">
         <v>12</v>
@@ -2686,13 +2608,13 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="B13" t="s">
         <v>3</v>
       </c>
       <c r="C13" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D13">
         <v>16.2</v>
@@ -2700,13 +2622,13 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B14" t="s">
         <v>2</v>
       </c>
       <c r="C14" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D14">
         <v>9.5</v>
@@ -2714,13 +2636,13 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B15" t="s">
         <v>2</v>
       </c>
       <c r="C15" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D15">
         <v>12.9</v>
@@ -2728,13 +2650,13 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B16" t="s">
         <v>2</v>
       </c>
       <c r="C16" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D16">
         <v>10.8</v>
@@ -2742,13 +2664,13 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B17" t="s">
         <v>2</v>
       </c>
       <c r="C17" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D17">
         <v>14.2</v>
@@ -2756,13 +2678,13 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B18" t="s">
         <v>2</v>
       </c>
       <c r="C18" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D18">
         <v>11.2</v>
@@ -2770,13 +2692,13 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B19" t="s">
         <v>2</v>
       </c>
       <c r="C19" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D19">
         <v>14.6</v>
@@ -2784,13 +2706,13 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B20" t="s">
         <v>2</v>
       </c>
       <c r="C20" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D20">
         <v>10.1</v>
@@ -2798,13 +2720,13 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B21" t="s">
         <v>2</v>
       </c>
       <c r="C21" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D21">
         <v>13.8</v>
@@ -2812,13 +2734,13 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B22" t="s">
         <v>2</v>
       </c>
       <c r="C22" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D22">
         <v>9.9</v>
@@ -2826,13 +2748,13 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B23" t="s">
         <v>2</v>
       </c>
       <c r="C23" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D23">
         <v>13.4</v>
@@ -2840,13 +2762,13 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B24" t="s">
         <v>2</v>
       </c>
       <c r="C24" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D24">
         <v>11.5</v>
@@ -2854,13 +2776,13 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B25" t="s">
         <v>2</v>
       </c>
       <c r="C25" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D25">
         <v>15</v>
@@ -2868,13 +2790,13 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="B26" t="s">
         <v>3</v>
       </c>
       <c r="C26" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D26">
         <v>10.7</v>
@@ -2882,13 +2804,13 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="B27" t="s">
         <v>3</v>
       </c>
       <c r="C27" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D27">
         <v>15.2</v>
@@ -2896,13 +2818,13 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B28" t="s">
         <v>3</v>
       </c>
       <c r="C28" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D28">
         <v>11.8</v>
@@ -2910,13 +2832,13 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B29" t="s">
         <v>3</v>
       </c>
       <c r="C29" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D29">
         <v>16.399999999999999</v>
@@ -2924,13 +2846,13 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B30" t="s">
         <v>3</v>
       </c>
       <c r="C30" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D30">
         <v>10.5</v>
@@ -2938,13 +2860,13 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="B31" t="s">
         <v>3</v>
       </c>
       <c r="C31" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D31">
         <v>14.9</v>
@@ -2952,13 +2874,13 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B32" t="s">
         <v>3</v>
       </c>
       <c r="C32" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D32">
         <v>12.3</v>
@@ -2966,13 +2888,13 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B33" t="s">
         <v>3</v>
       </c>
       <c r="C33" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D33">
         <v>16.8</v>
@@ -2980,13 +2902,13 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B34" t="s">
         <v>3</v>
       </c>
       <c r="C34" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D34">
         <v>11</v>
@@ -2994,13 +2916,13 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B35" t="s">
         <v>3</v>
       </c>
       <c r="C35" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D35">
         <v>15.6</v>
@@ -3008,13 +2930,13 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B36" t="s">
         <v>3</v>
       </c>
       <c r="C36" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D36">
         <v>12.2</v>
@@ -3022,13 +2944,13 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B37" t="s">
         <v>3</v>
       </c>
       <c r="C37" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D37">
         <v>16.5</v>
@@ -3036,13 +2958,13 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B38" t="s">
         <v>3</v>
       </c>
       <c r="C38" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D38">
         <v>11.3</v>
@@ -3050,13 +2972,13 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B39" t="s">
         <v>3</v>
       </c>
       <c r="C39" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D39">
         <v>15.1</v>
@@ -3064,13 +2986,13 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B40" t="s">
         <v>3</v>
       </c>
       <c r="C40" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D40">
         <v>10.9</v>
@@ -3078,13 +3000,13 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B41" t="s">
         <v>3</v>
       </c>
       <c r="C41" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D41">
         <v>15.3</v>
@@ -3108,215 +3030,374 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3CFCD11-B2BD-4FCD-AE43-A9AEC6806B3D}">
   <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="F1" s="11" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="9">
+        <v>0.32920625197414727</v>
+      </c>
+      <c r="C2" s="9">
+        <v>0.25616469835231498</v>
+      </c>
+      <c r="D2" s="9">
+        <v>0.30718435619652984</v>
+      </c>
+      <c r="E2" s="9">
+        <v>0.30264317645229644</v>
+      </c>
+      <c r="F2" s="12">
+        <v>0.43301627720466429</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="9">
+        <v>0.85398661071577375</v>
+      </c>
+      <c r="C3" s="9">
+        <v>0.86468452118538552</v>
+      </c>
+      <c r="D3" s="9">
+        <v>0.83745469859199428</v>
+      </c>
+      <c r="E3" s="9">
+        <v>0.93106232621453933</v>
+      </c>
+      <c r="F3" s="12">
+        <v>0.94661070517852552</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="9">
+        <v>1.1656312951809289</v>
+      </c>
+      <c r="C4" s="9">
+        <v>0.7186122785415</v>
+      </c>
+      <c r="D4" s="9">
+        <v>0.79120687522842825</v>
+      </c>
+      <c r="E4" s="9">
+        <v>1.4183153097242416</v>
+      </c>
+      <c r="F4" s="12">
+        <v>0.4715800213067059</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="9">
+        <v>1.1714611058888862</v>
+      </c>
+      <c r="C5" s="9">
+        <v>2.9750240825078458</v>
+      </c>
+      <c r="D5" s="9">
+        <v>2.2626430736689791</v>
+      </c>
+      <c r="E5" s="9">
+        <v>0.93230268428381813</v>
+      </c>
+      <c r="F5" s="12">
+        <v>2.2697742553538367</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" s="9">
+        <v>2.6049044104910708</v>
+      </c>
+      <c r="C6" s="9">
+        <v>2.1117276969504162</v>
+      </c>
+      <c r="D6" s="9">
+        <v>2.1713682272764845</v>
+      </c>
+      <c r="E6" s="9">
+        <v>2.6838647971351111</v>
+      </c>
+      <c r="F6" s="12">
+        <v>2.2792202931038061</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" s="9">
+        <v>131.93210530650757</v>
+      </c>
+      <c r="C7" s="9">
+        <v>6.5309583516666061</v>
+      </c>
+      <c r="D7" s="9">
+        <v>8.1921367456728813</v>
+      </c>
+      <c r="E7" s="9">
+        <v>5.1391410201983696</v>
+      </c>
+      <c r="F7" s="12">
+        <v>21.450873492178715</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" s="9">
+        <v>57.845577576799151</v>
+      </c>
+      <c r="C8" s="9">
+        <v>1.097962828599657</v>
+      </c>
+      <c r="D8" s="9">
+        <v>1.0477113070027784</v>
+      </c>
+      <c r="E8" s="9">
+        <v>2.1811559179243623</v>
+      </c>
+      <c r="F8" s="12">
+        <v>1.8741787135519767</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9" s="9">
+        <v>21.817022417933185</v>
+      </c>
+      <c r="C9" s="9">
+        <v>0.57239182310329562</v>
+      </c>
+      <c r="D9" s="9">
+        <v>0.89025038247988819</v>
+      </c>
+      <c r="E9" s="9">
+        <v>1.1889749520880042</v>
+      </c>
+      <c r="F9" s="12">
+        <v>2.2035834213797569</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="9">
+        <v>28.52252526579414</v>
+      </c>
+      <c r="C10" s="9">
+        <v>2.3279181954251946</v>
+      </c>
+      <c r="D10" s="10" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="E10" s="9">
+        <v>2.6635790712671299</v>
+      </c>
+      <c r="F10" s="12">
+        <v>2.6849291958847696</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" s="9">
+        <v>36.499140692051832</v>
+      </c>
+      <c r="C11" s="9">
+        <v>1.1525232791630275</v>
+      </c>
+      <c r="D11" s="9">
+        <v>1.629681948711277</v>
+      </c>
+      <c r="E11" s="9">
+        <v>1.7352515253585148</v>
+      </c>
+      <c r="F11" s="12">
+        <v>4.1331979713917981</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B2" s="5">
-        <v>562185.70700000005</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="B12" s="9">
+        <v>1.7771254469829192</v>
+      </c>
+      <c r="C12" s="9">
+        <v>0.56353930597080226</v>
+      </c>
+      <c r="D12" s="9">
+        <v>0.22847932329116452</v>
+      </c>
+      <c r="E12" s="9">
+        <v>0.10069961432961098</v>
+      </c>
+      <c r="F12" s="12">
+        <v>1.1868777416172649</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B3" s="5">
-        <v>556721.54099999997</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="B13" s="9">
+        <v>9.7956980672921841</v>
+      </c>
+      <c r="C13" s="9">
+        <v>0.51441269635792153</v>
+      </c>
+      <c r="D13" s="9">
+        <v>0.92571559963628924</v>
+      </c>
+      <c r="E13" s="9">
+        <v>0.76395046588380877</v>
+      </c>
+      <c r="F13" s="12">
+        <v>1.1083277347256366</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="5">
-        <v>495659.837</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+      <c r="B14" s="9">
+        <v>7.9767050884391839</v>
+      </c>
+      <c r="C14" s="9">
+        <v>0.37670173240110977</v>
+      </c>
+      <c r="D14" s="9">
+        <v>0.80784297177441111</v>
+      </c>
+      <c r="E14" s="9">
+        <v>0.80858617171502534</v>
+      </c>
+      <c r="F14" s="12">
+        <v>0.72512711387779338</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B5" s="5">
-        <v>494747.902</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+      <c r="B15" s="9">
+        <v>11.34678863730673</v>
+      </c>
+      <c r="C15" s="9">
+        <v>0.50714828602660111</v>
+      </c>
+      <c r="D15" s="9">
+        <v>0.51798242739061795</v>
+      </c>
+      <c r="E15" s="9">
+        <v>0.74876576496925296</v>
+      </c>
+      <c r="F15" s="12">
+        <v>1.0820087998705634</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B6" s="5">
-        <v>513508.70899999997</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="B7" s="5">
-        <v>325469.13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="B8" s="5">
-        <v>573058.84400000004</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="B9" s="5">
-        <v>541900.79299999995</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B10" s="5">
-        <v>423870.55599999998</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B11" s="5">
-        <v>414200.36499999999</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B12" s="5">
-        <v>506687.28399999999</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B13" s="5">
-        <v>377672.23300000001</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B14" s="5">
-        <v>237081.601</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B15" s="5">
-        <v>315259.571</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B16" s="5">
-        <v>275899.01199999999</v>
+      <c r="B16" s="9">
+        <v>7.8164145045059872</v>
+      </c>
+      <c r="C16" s="9">
+        <v>0.44794738922118515</v>
+      </c>
+      <c r="D16" s="9">
+        <v>0.5542780919645196</v>
+      </c>
+      <c r="E16" s="9">
+        <v>0.19714202083647198</v>
+      </c>
+      <c r="F16" s="12">
+        <v>1.4791269017769662</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B17" s="5">
-        <v>318830.84600000002</v>
-      </c>
+      <c r="A17" s="6"/>
+      <c r="B17" s="5"/>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B18" s="5">
-        <v>261227.54800000001</v>
-      </c>
+      <c r="A18" s="6"/>
+      <c r="B18" s="5"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B19" s="5">
-        <v>140315.93299999999</v>
-      </c>
+      <c r="A19" s="6"/>
+      <c r="B19" s="5"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B20" s="5">
-        <v>174263.75899999999</v>
-      </c>
+      <c r="A20" s="6"/>
+      <c r="B20" s="5"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B21" s="5">
-        <v>252005.19699999999</v>
-      </c>
+      <c r="A21" s="6"/>
+      <c r="B21" s="5"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B22" s="5">
-        <v>188084.73800000001</v>
-      </c>
+      <c r="A22" s="6"/>
+      <c r="B22" s="5"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B23" s="5">
-        <v>285774.902</v>
-      </c>
+      <c r="A23" s="6"/>
+      <c r="B23" s="5"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B24" s="5">
-        <v>239816.19500000001</v>
-      </c>
+      <c r="A24" s="6"/>
+      <c r="B24" s="5"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="B25" s="5">
-        <v>233596.87100000001</v>
-      </c>
+      <c r="A25" s="6"/>
+      <c r="B25" s="5"/>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="M29" s="6"/>

</xml_diff>

<commit_message>
Screenshots for the HowTo guide
</commit_message>
<xml_diff>
--- a/assets/StatisticalAnalyzer_Excel_Template.xlsx
+++ b/assets/StatisticalAnalyzer_Excel_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pkrumm\Documents\Statistik_dev\BioMedStatX---Code\assets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Philipp\Documents\BioMedStatX---Code\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51210420-C7EC-4F32-A0FE-9F4DADC3D4B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABA148A6-264B-487D-B34B-BCEACDF40195}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19320" yWindow="5985" windowWidth="19440" windowHeight="15000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="T-Test" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="57">
   <si>
     <t>Group</t>
   </si>
@@ -186,12 +186,6 @@
   </si>
   <si>
     <t>mPDL1 CNRQ</t>
-  </si>
-  <si>
-    <t>Gruppe</t>
-  </si>
-  <si>
-    <t>Messwert</t>
   </si>
   <si>
     <t>ntc</t>
@@ -256,6 +250,7 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -376,7 +371,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -679,7 +674,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -793,7 +788,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEFF587B-B563-4293-94E7-9E684D814310}">
   <dimension ref="A1:B73"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.5703125" customWidth="1"/>
     <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
@@ -801,10 +796,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>50</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -873,7 +868,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="15" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B10" s="14">
         <v>261227.54800000001</v>
@@ -881,7 +876,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="15" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B11" s="14">
         <v>140315.93299999999</v>
@@ -889,7 +884,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="15" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B12" s="14">
         <v>174263.75899999999</v>
@@ -897,7 +892,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="15" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B13" s="14">
         <v>252005.19699999999</v>
@@ -905,7 +900,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="15" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B14" s="14">
         <v>188084.73800000001</v>
@@ -913,7 +908,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="15" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B15" s="14">
         <v>285774.902</v>
@@ -921,7 +916,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="15" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B16" s="14">
         <v>239816.19500000001</v>
@@ -929,7 +924,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="15" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B17" s="14">
         <v>233596.87100000001</v>
@@ -937,7 +932,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="15" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B18" s="14">
         <v>351397.57799999998</v>
@@ -945,7 +940,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="15" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B19" s="14">
         <v>322996.69799999997</v>
@@ -953,7 +948,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="15" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B20" s="14">
         <v>211622.304</v>
@@ -961,7 +956,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="15" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B21" s="14">
         <v>566549.77099999995</v>
@@ -969,7 +964,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="15" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B22" s="14">
         <v>592641.29099999997</v>
@@ -977,7 +972,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="15" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B23" s="14">
         <v>673925.14199999999</v>
@@ -985,7 +980,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="15" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B24" s="14">
         <v>556283.74699999997</v>
@@ -993,7 +988,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="15" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B25" s="14">
         <v>593781.54099999997</v>
@@ -1001,7 +996,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="15" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B26" s="14">
         <v>562185.70700000005</v>
@@ -1009,7 +1004,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="15" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B27" s="14">
         <v>556721.54099999997</v>
@@ -1017,7 +1012,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="15" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B28" s="14">
         <v>495659.837</v>
@@ -1025,7 +1020,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="15" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B29" s="14">
         <v>494747.902</v>
@@ -1033,7 +1028,7 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="15" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B30" s="14">
         <v>513508.70899999997</v>
@@ -1041,7 +1036,7 @@
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="15" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B31" s="14">
         <v>325469.13</v>
@@ -1049,7 +1044,7 @@
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="15" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B32" s="14">
         <v>573058.84400000004</v>
@@ -1057,7 +1052,7 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="15" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B33" s="14">
         <v>541900.79299999995</v>
@@ -1065,7 +1060,7 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="13" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B34" s="14">
         <v>590576.53300000005</v>
@@ -1073,7 +1068,7 @@
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="13" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B35" s="14">
         <v>578878.00899999996</v>
@@ -1081,7 +1076,7 @@
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="13" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B36" s="14">
         <v>457073.26</v>
@@ -1089,7 +1084,7 @@
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="13" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B37" s="14">
         <v>423756.38699999999</v>
@@ -1097,7 +1092,7 @@
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="13" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B38" s="14">
         <v>305208.065</v>
@@ -1105,7 +1100,7 @@
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="13" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B39" s="14">
         <v>253590.75599999999</v>
@@ -1113,7 +1108,7 @@
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="13" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B40" s="14">
         <v>282297.69900000002</v>
@@ -1121,7 +1116,7 @@
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="13" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B41" s="14">
         <v>392604.62199999997</v>
@@ -1129,7 +1124,7 @@
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="13" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B42" s="14">
         <v>399257.95199999999</v>
@@ -1137,7 +1132,7 @@
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="13" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B43" s="14">
         <v>364420.76199999999</v>
@@ -1145,7 +1140,7 @@
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="13" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B44" s="14">
         <v>488414.43699999998</v>
@@ -1153,7 +1148,7 @@
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="13" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B45" s="14">
         <v>407326.261</v>
@@ -1161,7 +1156,7 @@
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="13" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B46" s="14">
         <v>239061.05</v>
@@ -1169,7 +1164,7 @@
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="13" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B47" s="14">
         <v>442695.326</v>
@@ -1177,7 +1172,7 @@
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="13" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B48" s="14">
         <v>427497.00699999998</v>
@@ -1185,7 +1180,7 @@
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="13" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B49" s="14">
         <v>505372.66</v>
@@ -1193,7 +1188,7 @@
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="13" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B50" s="14">
         <v>587377.82900000003</v>
@@ -1201,7 +1196,7 @@
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" s="13" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B51" s="14">
         <v>700124.54700000002</v>
@@ -1209,7 +1204,7 @@
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" s="13" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B52" s="14">
         <v>358138.73300000001</v>
@@ -1217,7 +1212,7 @@
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="13" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B53" s="14">
         <v>580047.09900000005</v>
@@ -1225,7 +1220,7 @@
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="13" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B54" s="14">
         <v>593144.28700000001</v>
@@ -1233,7 +1228,7 @@
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" s="13" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B55" s="14">
         <v>490447.81400000001</v>
@@ -1241,7 +1236,7 @@
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" s="13" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B56" s="14">
         <v>576824.54799999995</v>
@@ -1249,7 +1244,7 @@
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" s="13" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B57" s="14">
         <v>444891.76299999998</v>
@@ -1257,7 +1252,7 @@
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" s="13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B58" s="14">
         <v>435291.83899999998</v>
@@ -1265,7 +1260,7 @@
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" s="13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B59" s="14">
         <v>536366.39199999999</v>
@@ -1273,7 +1268,7 @@
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" s="13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B60" s="14">
         <v>516056.38799999998</v>
@@ -1281,7 +1276,7 @@
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" s="13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B61" s="14">
         <v>489389.109</v>
@@ -1289,7 +1284,7 @@
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" s="13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B62" s="14">
         <v>496422.53</v>
@@ -1297,7 +1292,7 @@
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" s="13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B63" s="14">
         <v>609042.57400000002</v>
@@ -1305,7 +1300,7 @@
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" s="13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B64" s="14">
         <v>460416.24200000003</v>
@@ -1313,7 +1308,7 @@
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="13" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B65" s="14">
         <v>510136.89600000001</v>
@@ -1321,7 +1316,7 @@
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="13" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B66" s="14">
         <v>423870.55599999998</v>
@@ -1329,7 +1324,7 @@
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="13" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B67" s="14">
         <v>414200.36499999999</v>
@@ -1337,7 +1332,7 @@
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" s="13" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B68" s="14">
         <v>506687.28399999999</v>
@@ -1345,7 +1340,7 @@
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" s="13" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B69" s="14">
         <v>377672.23300000001</v>
@@ -1353,7 +1348,7 @@
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" s="13" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B70" s="14">
         <v>237081.601</v>
@@ -1361,7 +1356,7 @@
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" s="13" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B71" s="14">
         <v>315259.571</v>
@@ -1369,7 +1364,7 @@
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" s="13" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B72" s="14">
         <v>275899.01199999999</v>
@@ -1377,7 +1372,7 @@
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" s="13" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B73" s="14">
         <v>318830.84600000002</v>
@@ -1391,7 +1386,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32BF23E1-8923-4AB2-B74C-427E6D1071D2}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -1490,7 +1485,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C28"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -1809,7 +1804,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE2D111A-A709-4CD9-B8AF-EA86CA23B91A}">
   <dimension ref="A1:C55"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7.85546875" bestFit="1" customWidth="1"/>
@@ -2430,7 +2425,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D43"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -3033,7 +3028,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3CFCD11-B2BD-4FCD-AE43-A9AEC6806B3D}">
   <dimension ref="A1:O29"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>

</xml_diff>